<commit_message>
fixed reports count sets
</commit_message>
<xml_diff>
--- a/data/uploads/malaria_report.xlsx
+++ b/data/uploads/malaria_report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/innocentwowa/Documents/Python Scripts/DashPlotly/data/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF34B275-F339-4045-844A-72ACE042C777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5974DCE-126C-C04F-98AE-4BCB515C2D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19880" activeTab="1" xr2:uid="{3D565A06-DCC6-034B-BC7E-69C7A268E9F5}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33860" windowHeight="19880" activeTab="1" xr2:uid="{3D565A06-DCC6-034B-BC7E-69C7A268E9F5}"/>
   </bookViews>
   <sheets>
     <sheet name="VARIABLE_NAMES" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="151">
   <si>
     <t>name</t>
   </si>
@@ -369,9 +369,6 @@
     <t>measure</t>
   </si>
   <si>
-    <t>count</t>
-  </si>
-  <si>
     <t>sum</t>
   </si>
   <si>
@@ -426,9 +423,6 @@
     <t>ASAQ 100mg/270mg (3 tablets) | ASAQ 100mg/270mg (6 tablets) | ASAQ 25mg/67.5mg (3 tablets) | ASAQ 50mg/135mg (3 tablets)</t>
   </si>
   <si>
-    <t>Malaria Species | Malaria film</t>
-  </si>
-  <si>
     <t>General</t>
   </si>
   <si>
@@ -453,38 +447,59 @@
     <t>programs</t>
   </si>
   <si>
-    <t>obs_value_coded | Value</t>
-  </si>
-  <si>
-    <t>Malaria | Positive</t>
-  </si>
-  <si>
     <t>Malaria</t>
   </si>
   <si>
-    <t>Patient pregnant | *diagnosis</t>
-  </si>
-  <si>
-    <t>concept_name | concept_name</t>
-  </si>
-  <si>
-    <t>obs_value_coded | obs_value_coded</t>
-  </si>
-  <si>
-    <t>Yes | Malaria</t>
-  </si>
-  <si>
     <t>malaria_total_under5</t>
   </si>
   <si>
     <t>malaria_total_over5</t>
+  </si>
+  <si>
+    <t>nunique</t>
+  </si>
+  <si>
+    <t>concept_name | Value</t>
+  </si>
+  <si>
+    <t>MRDT | Positive</t>
+  </si>
+  <si>
+    <t>concept_name | Value | obs_value_coded</t>
+  </si>
+  <si>
+    <t>MRDT | Positive | Malaria</t>
+  </si>
+  <si>
+    <t>MRDT | !=Positive | Malaria</t>
+  </si>
+  <si>
+    <t>MRDT | !=Positive</t>
+  </si>
+  <si>
+    <t>concept_name | concept_name | Value</t>
+  </si>
+  <si>
+    <t>Patient pregnant | MRDT | !=Positive</t>
+  </si>
+  <si>
+    <t>malaria_tx_failure_under5</t>
+  </si>
+  <si>
+    <t>malaria_tx_failure_over5</t>
+  </si>
+  <si>
+    <t>Malaria Treatment Failure</t>
+  </si>
+  <si>
+    <t>Malaria film</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -494,6 +509,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -519,11 +542,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -852,7 +876,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -887,10 +911,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C2" t="s">
         <v>39</v>
@@ -900,7 +924,7 @@
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
@@ -942,10 +966,10 @@
         <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D7" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -964,10 +988,10 @@
         <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>147</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
@@ -1071,18 +1095,18 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D20" t="s">
         <v>78</v>
@@ -1090,7 +1114,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" t="s">
         <v>79</v>
@@ -1098,7 +1122,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D22" t="s">
         <v>80</v>
@@ -1106,7 +1130,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D23" t="s">
         <v>81</v>
@@ -1114,7 +1138,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D24" t="s">
         <v>82</v>
@@ -1122,7 +1146,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D25" t="s">
         <v>83</v>
@@ -1130,7 +1154,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D26" t="s">
         <v>84</v>
@@ -1138,7 +1162,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
         <v>85</v>
@@ -1184,15 +1208,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420C8C5D-A000-9B41-8DCF-AB9A394A13A5}">
-  <dimension ref="A1:W39"/>
+  <dimension ref="A1:W41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" customWidth="1"/>
+    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="7" max="7" width="25.1640625" customWidth="1"/>
     <col min="8" max="8" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
@@ -1203,7 +1229,7 @@
         <v>108</v>
       </c>
       <c r="C1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D1" t="s">
         <v>13</v>
@@ -1271,28 +1297,34 @@
         <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H2" t="s">
         <v>37</v>
       </c>
       <c r="I2" t="s">
         <v>39</v>
+      </c>
+      <c r="J2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
@@ -1300,28 +1332,34 @@
         <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H3" t="s">
         <v>37</v>
       </c>
       <c r="I3" t="s">
-        <v>39</v>
+        <v>94</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
@@ -1329,28 +1367,34 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="G4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H4" t="s">
         <v>37</v>
       </c>
       <c r="I4" t="s">
         <v>39</v>
+      </c>
+      <c r="J4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
@@ -1358,28 +1402,34 @@
         <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="G5" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H5" t="s">
         <v>37</v>
       </c>
       <c r="I5" t="s">
         <v>94</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
@@ -1387,28 +1437,34 @@
         <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" t="s">
+        <v>94</v>
+      </c>
+      <c r="J6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" t="s">
         <v>135</v>
-      </c>
-      <c r="D6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E6" t="s">
-        <v>122</v>
-      </c>
-      <c r="F6" t="s">
-        <v>141</v>
-      </c>
-      <c r="G6" t="s">
-        <v>140</v>
-      </c>
-      <c r="H6" t="s">
-        <v>142</v>
-      </c>
-      <c r="I6" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
@@ -1416,51 +1472,57 @@
         <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F7" t="s">
+        <v>145</v>
+      </c>
+      <c r="G7" t="s">
+        <v>146</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" t="s">
         <v>135</v>
-      </c>
-      <c r="D7" t="s">
-        <v>123</v>
-      </c>
-      <c r="E7" t="s">
-        <v>122</v>
-      </c>
-      <c r="F7" t="s">
-        <v>141</v>
-      </c>
-      <c r="G7" t="s">
-        <v>140</v>
-      </c>
-      <c r="H7" t="s">
-        <v>142</v>
-      </c>
-      <c r="I7" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F8" t="s">
         <v>35</v>
       </c>
       <c r="G8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H8" t="s">
         <v>37</v>
@@ -1471,25 +1533,25 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F9" t="s">
         <v>35</v>
       </c>
       <c r="G9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H9" t="s">
         <v>37</v>
@@ -1503,16 +1565,16 @@
         <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H10" t="s">
         <v>37</v>
@@ -1526,16 +1588,16 @@
         <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H11" t="s">
         <v>37</v>
@@ -1546,25 +1608,25 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>147</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>149</v>
       </c>
       <c r="H12" t="s">
         <v>37</v>
@@ -1572,34 +1634,28 @@
       <c r="I12" t="s">
         <v>39</v>
       </c>
-      <c r="J12" t="s">
-        <v>96</v>
-      </c>
-      <c r="K12" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>149</v>
       </c>
       <c r="H13" t="s">
         <v>37</v>
@@ -1607,110 +1663,116 @@
       <c r="I13" t="s">
         <v>94</v>
       </c>
-      <c r="J13" t="s">
-        <v>96</v>
-      </c>
-      <c r="K13" t="s">
-        <v>126</v>
-      </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F14" t="s">
+        <v>141</v>
+      </c>
+      <c r="G14" t="s">
+        <v>142</v>
+      </c>
+      <c r="H14" t="s">
         <v>33</v>
       </c>
-      <c r="G14" t="s">
+      <c r="I14" t="s">
         <v>95</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>37</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>39</v>
       </c>
-      <c r="J14" t="s">
+      <c r="L14" t="s">
         <v>96</v>
       </c>
-      <c r="K14" t="s">
-        <v>127</v>
+      <c r="M14" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F15" t="s">
+        <v>141</v>
+      </c>
+      <c r="G15" t="s">
+        <v>142</v>
+      </c>
+      <c r="H15" t="s">
         <v>33</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
         <v>95</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>37</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>94</v>
       </c>
-      <c r="J15" t="s">
+      <c r="L15" t="s">
         <v>96</v>
       </c>
-      <c r="K15" t="s">
-        <v>127</v>
+      <c r="M15" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F16" t="s">
+        <v>141</v>
+      </c>
+      <c r="G16" t="s">
+        <v>143</v>
+      </c>
+      <c r="H16" t="s">
         <v>33</v>
       </c>
-      <c r="G16" t="s">
-        <v>97</v>
-      </c>
-      <c r="H16" t="s">
-        <v>34</v>
-      </c>
       <c r="I16" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="J16" t="s">
         <v>37</v>
@@ -1718,34 +1780,40 @@
       <c r="K16" t="s">
         <v>39</v>
       </c>
+      <c r="L16" t="s">
+        <v>96</v>
+      </c>
+      <c r="M16" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B17" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="C17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F17" t="s">
+        <v>141</v>
+      </c>
+      <c r="G17" t="s">
+        <v>143</v>
+      </c>
+      <c r="H17" t="s">
         <v>33</v>
       </c>
-      <c r="G17" t="s">
-        <v>97</v>
-      </c>
-      <c r="H17" t="s">
-        <v>34</v>
-      </c>
       <c r="I17" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="J17" t="s">
         <v>37</v>
@@ -1753,22 +1821,28 @@
       <c r="K17" t="s">
         <v>94</v>
       </c>
+      <c r="L17" t="s">
+        <v>96</v>
+      </c>
+      <c r="M17" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F18" t="s">
         <v>33</v>
@@ -1783,33 +1857,27 @@
         <v>98</v>
       </c>
       <c r="J18" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="K18" t="s">
-        <v>100</v>
-      </c>
-      <c r="L18" t="s">
-        <v>37</v>
-      </c>
-      <c r="M18" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F19" t="s">
         <v>33</v>
@@ -1824,33 +1892,27 @@
         <v>98</v>
       </c>
       <c r="J19" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="K19" t="s">
-        <v>100</v>
-      </c>
-      <c r="L19" t="s">
-        <v>37</v>
-      </c>
-      <c r="M19" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E20" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F20" t="s">
         <v>33</v>
@@ -1862,30 +1924,36 @@
         <v>34</v>
       </c>
       <c r="I20" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
       <c r="J20" t="s">
+        <v>99</v>
+      </c>
+      <c r="K20" t="s">
+        <v>100</v>
+      </c>
+      <c r="L20" t="s">
         <v>37</v>
       </c>
-      <c r="K20" t="s">
+      <c r="M20" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C21" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F21" t="s">
         <v>33</v>
@@ -1897,30 +1965,36 @@
         <v>34</v>
       </c>
       <c r="I21" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
       <c r="J21" t="s">
+        <v>99</v>
+      </c>
+      <c r="K21" t="s">
+        <v>100</v>
+      </c>
+      <c r="L21" t="s">
         <v>37</v>
       </c>
-      <c r="K21" t="s">
+      <c r="M21" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C22" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F22" t="s">
         <v>33</v>
@@ -1932,36 +2006,30 @@
         <v>34</v>
       </c>
       <c r="I22" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="J22" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="K22" t="s">
-        <v>100</v>
-      </c>
-      <c r="L22" t="s">
-        <v>37</v>
-      </c>
-      <c r="M22" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B23" t="s">
-        <v>109</v>
+        <v>138</v>
       </c>
       <c r="C23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F23" t="s">
         <v>33</v>
@@ -1973,94 +2041,112 @@
         <v>34</v>
       </c>
       <c r="I23" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="J23" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="K23" t="s">
-        <v>100</v>
-      </c>
-      <c r="L23" t="s">
-        <v>37</v>
-      </c>
-      <c r="M23" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B24" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D24" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F24" t="s">
         <v>33</v>
       </c>
       <c r="G24" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H24" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="I24" t="s">
-        <v>101</v>
+        <v>150</v>
+      </c>
+      <c r="J24" t="s">
+        <v>99</v>
+      </c>
+      <c r="K24" t="s">
+        <v>100</v>
+      </c>
+      <c r="L24" t="s">
+        <v>37</v>
+      </c>
+      <c r="M24" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
       <c r="C25" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F25" t="s">
         <v>33</v>
       </c>
       <c r="G25" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H25" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="I25" t="s">
-        <v>102</v>
+        <v>150</v>
+      </c>
+      <c r="J25" t="s">
+        <v>99</v>
+      </c>
+      <c r="K25" t="s">
+        <v>100</v>
+      </c>
+      <c r="L25" t="s">
+        <v>37</v>
+      </c>
+      <c r="M25" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C26" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F26" t="s">
         <v>33</v>
@@ -2072,24 +2158,24 @@
         <v>96</v>
       </c>
       <c r="I26" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D27" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F27" t="s">
         <v>33</v>
@@ -2101,24 +2187,24 @@
         <v>96</v>
       </c>
       <c r="I27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B28" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C28" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F28" t="s">
         <v>33</v>
@@ -2130,24 +2216,24 @@
         <v>96</v>
       </c>
       <c r="I28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D29" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E29" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F29" t="s">
         <v>33</v>
@@ -2159,30 +2245,24 @@
         <v>96</v>
       </c>
       <c r="I29" t="s">
-        <v>105</v>
-      </c>
-      <c r="J29" t="s">
-        <v>37</v>
-      </c>
-      <c r="K29" t="s">
-        <v>39</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C30" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D30" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F30" t="s">
         <v>33</v>
@@ -2199,19 +2279,19 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D31" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E31" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F31" t="s">
         <v>33</v>
@@ -2223,24 +2303,30 @@
         <v>96</v>
       </c>
       <c r="I31" t="s">
-        <v>98</v>
+        <v>105</v>
+      </c>
+      <c r="J31" t="s">
+        <v>37</v>
+      </c>
+      <c r="K31" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E32" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F32" t="s">
         <v>33</v>
@@ -2252,24 +2338,24 @@
         <v>96</v>
       </c>
       <c r="I32" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B33" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D33" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E33" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F33" t="s">
         <v>33</v>
@@ -2281,24 +2367,24 @@
         <v>96</v>
       </c>
       <c r="I33" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B34" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C34" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D34" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F34" t="s">
         <v>33</v>
@@ -2310,24 +2396,24 @@
         <v>96</v>
       </c>
       <c r="I34" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C35" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D35" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F35" t="s">
         <v>33</v>
@@ -2339,11 +2425,69 @@
         <v>96</v>
       </c>
       <c r="I35" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" t="s">
+        <v>111</v>
+      </c>
+      <c r="D36" t="s">
+        <v>122</v>
+      </c>
+      <c r="E36" t="s">
+        <v>121</v>
+      </c>
+      <c r="F36" t="s">
+        <v>33</v>
+      </c>
+      <c r="G36" t="s">
+        <v>95</v>
+      </c>
+      <c r="H36" t="s">
+        <v>96</v>
+      </c>
+      <c r="I36" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C37" t="s">
+        <v>111</v>
+      </c>
+      <c r="D37" t="s">
+        <v>122</v>
+      </c>
+      <c r="E37" t="s">
+        <v>121</v>
+      </c>
+      <c r="F37" t="s">
+        <v>33</v>
+      </c>
+      <c r="G37" t="s">
+        <v>95</v>
+      </c>
+      <c r="H37" t="s">
+        <v>96</v>
+      </c>
+      <c r="I37" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J39" s="1"/>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J41" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2368,7 +2512,7 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2376,10 +2520,10 @@
         <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2432,7 +2576,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
merged datafix x reporting fix
</commit_message>
<xml_diff>
--- a/data/uploads/malaria_report.xlsx
+++ b/data/uploads/malaria_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/innocentwowa/Documents/Python Scripts/DashPlotly/data/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A643E14-D666-9D45-A24B-42F541C8D546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B9EB9E-7013-1E44-A595-2A2B1F967CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="33860" windowHeight="19880" activeTab="1" xr2:uid="{3D565A06-DCC6-034B-BC7E-69C7A268E9F5}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="SETTINGS" sheetId="4" r:id="rId4"/>
     <sheet name="DESIGN" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
fixed dhis integrater params and count_sets
</commit_message>
<xml_diff>
--- a/data/uploads/malaria_report.xlsx
+++ b/data/uploads/malaria_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/innocentwowa/Documents/Python Scripts/DashPlotly/data/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B9EB9E-7013-1E44-A595-2A2B1F967CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B3B6F60-ADE2-0046-8B08-0BEC4BAD7D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="33860" windowHeight="19880" activeTab="1" xr2:uid="{3D565A06-DCC6-034B-BC7E-69C7A268E9F5}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="152">
   <si>
     <t>name</t>
   </si>
@@ -493,6 +493,9 @@
   </si>
   <si>
     <t>Malaria film</t>
+  </si>
+  <si>
+    <t>Malaria | Malaria</t>
   </si>
 </sst>
 </file>
@@ -1324,7 +1327,7 @@
         <v>35</v>
       </c>
       <c r="K2" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">

</xml_diff>